<commit_message>
Add Search part 2
</commit_message>
<xml_diff>
--- a/wooclap/imports/04_Search_Part_2.xlsx
+++ b/wooclap/imports/04_Search_Part_2.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>L01-C06 · A journey has cost 4 so far. You estimate that the remaining journey will cost 3. What is your estimate of the total cost?</t>
+          <t>L01-C06 · The frontier contains paths P, Q and R. Their costs so far g and remaining estimates h are: P (6, 1), Q (2, 4), R (4, 3). Greedy selects minimum h; A* selects minimum g + h. Which paths do they select next?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -530,22 +530,22 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>1.</t>
+          <t>Both select P, because its remaining estimate is smallest.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>3.</t>
+          <t>Both select Q, because its cost so far is smallest.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>7.</t>
+          <t>Greedy selects P; A* selects Q, whose total estimate is 6.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>4.</t>
+          <t>Greedy selects P; A* ties P and R at a total estimate of 7.</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
@@ -560,7 +560,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>L01-C07 · A search finds a cheaper route to a place it has already reached. What information should it keep?</t>
+          <t>L01-C07 · Graph A* has expanded X at cost g = 6 and found X→G with cost 3. Later it finds a route to X at g = 4. Its heuristic is admissible but inconsistent; G is the goal. Which action preserves the cheaper route through X?</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -570,22 +570,22 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Only the first route, even when it is more expensive.</t>
+          <t>Keep X closed: an admissible heuristic makes its first expansion final.</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Only the name of the place, with no cost information.</t>
+          <t>Update X to g = 4, but do not revisit its outgoing edge; keep G at cost 9.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>A claim that no route to this place exists.</t>
+          <t>Reopen X at g = 4, but keep G at cost 9 because a goal was already discovered.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>The new, lower cost and the route that achieves it.</t>
+          <t>Update X’s cost and parent, reopen it, and propagate the improvement to G at cost 7.</t>
         </is>
       </c>
       <c r="H3" s="3" t="n"/>
@@ -600,7 +600,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>L01-C08 · Your best complete route costs 6. Another route already costs 8, and every extra step adds a nonnegative cost. Can it beat your best route?</t>
+          <t>L01-C08 · Branch-and-bound already holds a complete route costing 6. Waiting path P has g = 4, h = 3; Q has g = 2, h = 4. The estimates are admissible and costs nonnegative. If the aim is to return one cheapest route, which paths may be pruned?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -610,22 +610,22 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Yes. Taking more steps always makes a route cheaper.</t>
+          <t>Only P: a lower bound equal to 6 must always be explored.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Yes. An unfinished route always beats a finished one.</t>
+          <t>Only Q: its remaining estimate is larger than P’s.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>No. Continuing cannot bring its total below 6.</t>
+          <t>Both P and Q: neither lower bound is below 6, and the saved route is retained.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>There is not enough information, even with the stated cost rule.</t>
+          <t>Neither: their costs so far are below 6, so both must be completed.</t>
         </is>
       </c>
       <c r="H4" s="2" t="n"/>
@@ -640,7 +640,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>L01-C09 · In one sentence, explain the main difference between breadth-first and depth-first search.</t>
+          <t>L01-C09 · A graph A* search uses an admissible but inconsistent heuristic and never reopens expanded states. Can its first selected goal be suboptimal? Explain using the reopening example, where cost 6 improves to 5, and state the repair.</t>
         </is>
       </c>
       <c r="C5" s="3" t="n"/>

</xml_diff>